<commit_message>
Publish v0.1.1 verified IBC and lead-lag corrections
</commit_message>
<xml_diff>
--- a/outputs/atom_flash_crash_2025_10_10/cosmoshub_flow_analysis.xlsx
+++ b/outputs/atom_flash_crash_2025_10_10/cosmoshub_flow_analysis.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R77865f85e91643c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Summary" sheetId="2" r:id="R8a0e9491c3464bc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Controls" sheetId="3" r:id="Re6d041fda9914be0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Dist" sheetId="4" r:id="Rcedec5d5881b4243"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Periods" sheetId="5" r:id="R6c7a641adf6c4677"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="6" r:id="R9a1e903356af4f7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidates" sheetId="7" r:id="Rd27b29f0635543bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IBC Routes" sheetId="8" r:id="R882c4d097a7c41e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5min Series" sheetId="9" r:id="R5212f5b66d6340c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="10" r:id="R5e6a223bee2b468c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30d Tests" sheetId="11" r:id="Rc4d7201f64d3403b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30d Controls" sheetId="12" r:id="R6a204c6e932d47eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Lag" sheetId="13" r:id="Raf142bd4dede41bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lag Curves" sheetId="14" r:id="R68bec3d73e8e4a02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robustness" sheetId="15" r:id="R4154a45c53024651"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R940a7ea73b484cb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Summary" sheetId="2" r:id="Rdb365e0aab0d450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Controls" sheetId="3" r:id="R3b21494557e64218"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Dist" sheetId="4" r:id="R4672ab37f7914293"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Periods" sheetId="5" r:id="R3cd087608c8d453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="6" r:id="R716c9924cac841f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidates" sheetId="7" r:id="Ra9ccb1b66b944866"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IBC Routes" sheetId="8" r:id="Rf7e326953e9e45bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5min Series" sheetId="9" r:id="Rd2d3d52418084b87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="10" r:id="Rd34df91010744a3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30d Tests" sheetId="11" r:id="R02c33eb7788c47ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30d Controls" sheetId="12" r:id="R21b14c8d7f5a4490"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Lag" sheetId="13" r:id="Re65a766ac97b4c93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lag Curves" sheetId="14" r:id="R6d66531763e34763"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robustness" sheetId="15" r:id="R08308f4f7d564654"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -250,7 +250,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="13">
+  <x:dxfs count="17">
     <x:dxf>
       <x:font>
         <x:color rgb="FFB91C1C"/>
@@ -295,6 +295,46 @@
       <x:font>
         <x:color rgb="FFB91C1C"/>
       </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4DF"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF0F766E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7F6F3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFD97706"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4DF"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF0F766E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7F6F3"/>
+        </x:patternFill>
+      </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
@@ -1450,7 +1490,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra7a5e465dcd84917"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R81e394f5a41d412c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1485,7 +1525,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6c2dfb3346ba424d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb3a07b758a5148a7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1520,7 +1560,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc030805a1d1945a4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R17dd3f3f081043d9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1555,7 +1595,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R28af2cf43362497d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R790789e75251444f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1590,7 +1630,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6e27ac45c7a74d1d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc7fe90d3dfb040cb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2003,7 +2043,7 @@
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
       <x:c r="A17" s="49" t="str">
-        <x:v>Against 360 pre-event two-hour windows, the Binance ATOM/USDT range was at the 100.0th empirical percentile (p=0.0028). Confirmed-label exchange inflow was 188,053.42 ATOM (93.9th percentile; p=0.0637), while confirmed plus unconfirmed behavioral candidates totaled 1,582,053.197 ATOM (p=0.0139). IBC outbound was 450,890.178 ATOM (p=0.0139). Primary inference uses only four public-record labels. Without historical Binance order-book snapshots, the pattern is consistent with a pair-specific liquidity or market-microstructure disruption, but does not prove liquidity depletion.</x:v>
+        <x:v>Against 360 pre-event two-hour windows, the Binance ATOM/USDT range was at the 100.0th empirical percentile (p=0.0028). Exact-match exchange inflow was 188,053.42 ATOM (93.9th percentile; p=0.0637), while exact-match plus unconfirmed candidates totaled 1,582,053.197 ATOM (p=0.0139). IBC outbound was 450,890.178 ATOM (p=0.0139). These probabilities describe baseline rarity under serial dependence. Public labels do not verify beneficial ownership. Without historical Binance order books, the pattern is consistent with pair-specific microstructure disruption, not proof of liquidity depletion.</x:v>
       </x:c>
       <x:c r="B17" s="49"/>
       <x:c r="C17" s="49"/>
@@ -2067,7 +2107,7 @@
         <x:v>Methods sheet</x:v>
       </x:c>
       <x:c r="D24" s="13" t="str">
-        <x:v>34,770 IBC transfers extracted</x:v>
+        <x:v>34,760 IBC transfers extracted</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="21" customHeight="1">
@@ -2109,7 +2149,7 @@
         <x:v>Methods sheet</x:v>
       </x:c>
       <x:c r="D27" s="13" t="str">
-        <x:v>Exact 2025-10-09 overlap reconciliation</x:v>
+        <x:v>Receipt-v2 baseline and exact 2025-10-09 overlap reconciliation</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="21" customHeight="1">
@@ -2123,7 +2163,7 @@
         <x:v>Methods sheet</x:v>
       </x:c>
       <x:c r="D28" s="52" t="str">
-        <x:v>Window tests and lead-lag extrema independently recalculated</x:v>
+        <x:v>Window tests and matched-statistic circular shifts recalculated</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2876,7 +2916,7 @@
     <x:mergeCell ref="A17:D20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81d1f5b604e04517"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc7f0243850041da"/>
 </x:worksheet>
 </file>
 
@@ -2938,7 +2978,7 @@
         <x:v>IBC transfers</x:v>
       </x:c>
       <x:c r="B5" s="51" t="str">
-        <x:v>Successful ICS-20 send/receive packet data; inbound native ATOM recognized by */uatom path</x:v>
+        <x:v>IBC inbound requires matching application success, native-return trace and native uatom credit, including forwarding intermediary credit. Outbound records successful Hub send initiation, not final destination settlement.</x:v>
       </x:c>
       <x:c r="C5" s="51" t="str">
         <x:v>data/processed/cosmoshub/ibc_transfers_2025-10-09_2025-10-12.jsonl.gz</x:v>
@@ -3023,10 +3063,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="51" t="str">
-        <x:v>Main randomization set</x:v>
+        <x:v>Main empirical reference set</x:v>
       </x:c>
       <x:c r="B13" s="51" t="str">
-        <x:v>360 non-overlapping UTC-aligned two-hour windows; plus-one exact rank/randomization p-values</x:v>
+        <x:v>360 non-overlapping UTC-aligned two-hour windows; plus-one probabilities describe baseline rarity, not exact randomization significance under serial dependence.</x:v>
       </x:c>
       <x:c r="C13" s="51" t="str">
         <x:v>results/publication_additional_analysis.json</x:v>
@@ -3070,7 +3110,7 @@
         <x:v>Lead-lag significance</x:v>
       </x:c>
       <x:c r="B17" s="51" t="str">
-        <x:v>Circular-shift max-|correlation| test across all reported lags, deterministic seed 20251010</x:v>
+        <x:v>Circular-shift max-|Pearson correlation| uses identical finite-pair, lag-trimmed normalization for observed and shifted samples; deterministic seed 20251010.</x:v>
       </x:c>
       <x:c r="C17" s="51" t="str">
         <x:v>results/publication_additional_analysis.json</x:v>
@@ -3103,7 +3143,7 @@
         <x:v>30-day Cosmos verification</x:v>
       </x:c>
       <x:c r="B20" s="51" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PASS: receipt-v2 manifest, source hashes and overlap reconciled</x:v>
       </x:c>
       <x:c r="C20" s="51" t="str">
         <x:v>results/cosmos_baseline_30d_verification.json</x:v>
@@ -3114,7 +3154,7 @@
         <x:v>Publication statistics verification</x:v>
       </x:c>
       <x:c r="B21" s="51" t="str">
-        <x:v>PASS</x:v>
+        <x:v>PASS: window tables and independent primary Pearson circular shifts</x:v>
       </x:c>
       <x:c r="C21" s="51" t="str">
         <x:v>results/publication_additional_verification.json</x:v>
@@ -3164,7 +3204,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="20" t="str">
-        <x:v>Thirty-day event-window rank and randomization tests</x:v>
+        <x:v>Thirty-day event-window ranks and empirical tail probabilities</x:v>
       </x:c>
       <x:c r="B1" s="20"/>
       <x:c r="C1" s="20"/>
@@ -3845,7 +3885,7 @@
       </x:c>
       <x:c r="G17" s="15" t="n">
         <x:f>AVERAGE('30d Controls'!$J$2:$J$361)</x:f>
-        <x:v>28023.37552831944</x:v>
+        <x:v>28022.782008666665</x:v>
       </x:c>
       <x:c r="H17" s="15" t="n">
         <x:f>MEDIAN('30d Controls'!$J$2:$J$361)</x:f>
@@ -3894,7 +3934,7 @@
       </x:c>
       <x:c r="G18" s="15" t="n">
         <x:f>AVERAGE('30d Controls'!$J$362:$J$391)</x:f>
-        <x:v>51032.05203786667</x:v>
+        <x:v>51031.26016869999</x:v>
       </x:c>
       <x:c r="H18" s="15" t="n">
         <x:f>MEDIAN('30d Controls'!$J$362:$J$391)</x:f>
@@ -4041,7 +4081,7 @@
       </x:c>
       <x:c r="G21" s="15" t="n">
         <x:f>AVERAGE('30d Controls'!$L$2:$L$361)</x:f>
-        <x:v>68465.2927329111</x:v>
+        <x:v>68464.69921325833</x:v>
       </x:c>
       <x:c r="H21" s="15" t="n">
         <x:f>MEDIAN('30d Controls'!$L$2:$L$361)</x:f>
@@ -4090,7 +4130,7 @@
       </x:c>
       <x:c r="G22" s="15" t="n">
         <x:f>AVERAGE('30d Controls'!$L$362:$L$391)</x:f>
-        <x:v>128576.70098626669</x:v>
+        <x:v>128575.90911710003</x:v>
       </x:c>
       <x:c r="H22" s="15" t="n">
         <x:f>MEDIAN('30d Controls'!$L$362:$L$391)</x:f>
@@ -4102,7 +4142,7 @@
       </x:c>
       <x:c r="J22" s="15" t="n">
         <x:f>SMALL('30d Controls'!$L$362:$L$391,MAX(1,ROUNDUP(F22*0.95,0)))</x:f>
-        <x:v>217814.206915</x:v>
+        <x:v>217790.45084</x:v>
       </x:c>
       <x:c r="K22" s="22" t="n">
         <x:f>COUNTIF('30d Controls'!$L$362:$L$391,"&lt;="&amp;E22)/F22</x:f>
@@ -4139,7 +4179,7 @@
       </x:c>
       <x:c r="G23" s="15" t="n">
         <x:f>AVERAGE('30d Controls'!$M$2:$M$361)</x:f>
-        <x:v>-12418.54167627222</x:v>
+        <x:v>-12419.135195924999</x:v>
       </x:c>
       <x:c r="H23" s="15" t="n">
         <x:f>MEDIAN('30d Controls'!$M$2:$M$361)</x:f>
@@ -4147,7 +4187,7 @@
       </x:c>
       <x:c r="I23" s="15" t="n">
         <x:f>SMALL('30d Controls'!$M$2:$M$361,MAX(1,ROUNDUP(F23*0.05,0)))</x:f>
-        <x:v>-42636.434010000004</x:v>
+        <x:v>-42776.05201000001</x:v>
       </x:c>
       <x:c r="J23" s="15" t="n">
         <x:f>SMALL('30d Controls'!$M$2:$M$361,MAX(1,ROUNDUP(F23*0.95,0)))</x:f>
@@ -4188,7 +4228,7 @@
       </x:c>
       <x:c r="G24" s="15" t="n">
         <x:f>AVERAGE('30d Controls'!$M$362:$M$391)</x:f>
-        <x:v>-26512.59691053333</x:v>
+        <x:v>-26513.388779700002</x:v>
       </x:c>
       <x:c r="H24" s="15" t="n">
         <x:f>MEDIAN('30d Controls'!$M$362:$M$391)</x:f>
@@ -4196,7 +4236,7 @@
       </x:c>
       <x:c r="I24" s="15" t="n">
         <x:f>SMALL('30d Controls'!$M$362:$M$391,MAX(1,ROUNDUP(F24*0.05,0)))</x:f>
-        <x:v>-168803.251095</x:v>
+        <x:v>-168827.00717</x:v>
       </x:c>
       <x:c r="J24" s="15" t="n">
         <x:f>SMALL('30d Controls'!$M$362:$M$391,MAX(1,ROUNDUP(F24*0.95,0)))</x:f>
@@ -5004,12 +5044,12 @@
     <x:mergeCell ref="A1:M2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="M5:M40">
-    <x:cfRule type="cellIs" dxfId="10" priority="1" operator="lessThanOrEqual">
+    <x:cfRule type="cellIs" dxfId="14" priority="1" operator="lessThanOrEqual">
       <x:formula>0.05</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="K5:K40">
-    <x:cfRule type="cellIs" dxfId="11" priority="2" operator="greaterThanOrEqual">
+    <x:cfRule type="cellIs" dxfId="15" priority="2" operator="greaterThanOrEqual">
       <x:formula>0.95</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -10728,16 +10768,16 @@
         <x:v>53408.680282</x:v>
       </x:c>
       <x:c r="J88" s="15" t="n">
-        <x:v>1949.604597</x:v>
+        <x:v>1944.932597</x:v>
       </x:c>
       <x:c r="K88" s="15" t="n">
         <x:v>7620.718771</x:v>
       </x:c>
       <x:c r="L88" s="15" t="n">
-        <x:v>9570.323368</x:v>
+        <x:v>9565.651367999999</x:v>
       </x:c>
       <x:c r="M88" s="15" t="n">
-        <x:v>-5671.114174</x:v>
+        <x:v>-5675.786174</x:v>
       </x:c>
       <x:c r="N88" s="15" t="n">
         <x:v>0.9513274336283221</x:v>
@@ -19048,16 +19088,16 @@
         <x:v>234216.91739900003</x:v>
       </x:c>
       <x:c r="J216" s="15" t="n">
-        <x:v>21359.052639</x:v>
+        <x:v>21335.296564</x:v>
       </x:c>
       <x:c r="K216" s="15" t="n">
         <x:v>197020.913687</x:v>
       </x:c>
       <x:c r="L216" s="15" t="n">
-        <x:v>218379.966326</x:v>
+        <x:v>218356.21025099998</x:v>
       </x:c>
       <x:c r="M216" s="15" t="n">
-        <x:v>-175661.861048</x:v>
+        <x:v>-175685.617123</x:v>
       </x:c>
       <x:c r="N216" s="15" t="n">
         <x:v>1.3245033112582847</x:v>
@@ -22298,16 +22338,16 @@
         <x:v>457266.67679</x:v>
       </x:c>
       <x:c r="J266" s="15" t="n">
-        <x:v>140234.149413</x:v>
+        <x:v>140227.784413</x:v>
       </x:c>
       <x:c r="K266" s="15" t="n">
         <x:v>24229.346192999998</x:v>
       </x:c>
       <x:c r="L266" s="15" t="n">
-        <x:v>164463.495606</x:v>
+        <x:v>164457.130606</x:v>
       </x:c>
       <x:c r="M266" s="15" t="n">
-        <x:v>116004.80322</x:v>
+        <x:v>115998.43821999998</x:v>
       </x:c>
       <x:c r="N266" s="15" t="n">
         <x:v>1.812907904278467</x:v>
@@ -22493,16 +22533,16 @@
         <x:v>99840.06076</x:v>
       </x:c>
       <x:c r="J269" s="15" t="n">
-        <x:v>23774.471319</x:v>
+        <x:v>23768.105319</x:v>
       </x:c>
       <x:c r="K269" s="15" t="n">
         <x:v>41564.760129</x:v>
       </x:c>
       <x:c r="L269" s="15" t="n">
-        <x:v>65339.231448000006</x:v>
+        <x:v>65332.865448</x:v>
       </x:c>
       <x:c r="M269" s="15" t="n">
-        <x:v>-17790.288810000002</x:v>
+        <x:v>-17796.654810000004</x:v>
       </x:c>
       <x:c r="N269" s="15" t="n">
         <x:v>0.8074091664687677</x:v>
@@ -23078,16 +23118,16 @@
         <x:v>97907.80789699999</x:v>
       </x:c>
       <x:c r="J278" s="15" t="n">
-        <x:v>19949.985322</x:v>
+        <x:v>19943.615322</x:v>
       </x:c>
       <x:c r="K278" s="15" t="n">
         <x:v>25104.830141000002</x:v>
       </x:c>
       <x:c r="L278" s="15" t="n">
-        <x:v>45054.815463000006</x:v>
+        <x:v>45048.445463000004</x:v>
       </x:c>
       <x:c r="M278" s="15" t="n">
-        <x:v>-5154.844819000002</x:v>
+        <x:v>-5161.214819000001</x:v>
       </x:c>
       <x:c r="N278" s="15" t="n">
         <x:v>2.109411219286029</x:v>
@@ -23858,16 +23898,16 @@
         <x:v>148580.41336</x:v>
       </x:c>
       <x:c r="J290" s="15" t="n">
-        <x:v>26100.570715</x:v>
+        <x:v>26094.198715</x:v>
       </x:c>
       <x:c r="K290" s="15" t="n">
         <x:v>26107.176071</x:v>
       </x:c>
       <x:c r="L290" s="15" t="n">
-        <x:v>52207.746786</x:v>
+        <x:v>52201.374786</x:v>
       </x:c>
       <x:c r="M290" s="15" t="n">
-        <x:v>-6.605356000000029</x:v>
+        <x:v>-12.977356000003056</x:v>
       </x:c>
       <x:c r="N290" s="15" t="n">
         <x:v>1.4018691588785164</x:v>
@@ -24638,16 +24678,16 @@
         <x:v>112246.210127</x:v>
       </x:c>
       <x:c r="J302" s="15" t="n">
-        <x:v>3534.170104</x:v>
+        <x:v>3527.798104</x:v>
       </x:c>
       <x:c r="K302" s="15" t="n">
         <x:v>2848.646104</x:v>
       </x:c>
       <x:c r="L302" s="15" t="n">
-        <x:v>6382.816208</x:v>
+        <x:v>6376.444208</x:v>
       </x:c>
       <x:c r="M302" s="15" t="n">
-        <x:v>685.5239999999999</x:v>
+        <x:v>679.152</x:v>
       </x:c>
       <x:c r="N302" s="15" t="n">
         <x:v>0.8220502901353918</x:v>
@@ -25418,16 +25458,16 @@
         <x:v>142709.357236</x:v>
       </x:c>
       <x:c r="J314" s="15" t="n">
-        <x:v>28393.708903000002</x:v>
+        <x:v>28387.328903</x:v>
       </x:c>
       <x:c r="K314" s="15" t="n">
         <x:v>38100.293628</x:v>
       </x:c>
       <x:c r="L314" s="15" t="n">
-        <x:v>66494.002531</x:v>
+        <x:v>66487.622531</x:v>
       </x:c>
       <x:c r="M314" s="15" t="n">
-        <x:v>-9706.584724999997</x:v>
+        <x:v>-9712.964724999998</x:v>
       </x:c>
       <x:c r="N314" s="15" t="n">
         <x:v>1.591128254580517</x:v>
@@ -25613,16 +25653,16 @@
         <x:v>110668.607142</x:v>
       </x:c>
       <x:c r="J317" s="15" t="n">
-        <x:v>42031.809371</x:v>
+        <x:v>41892.191371</x:v>
       </x:c>
       <x:c r="K317" s="15" t="n">
         <x:v>84668.24338100001</x:v>
       </x:c>
       <x:c r="L317" s="15" t="n">
-        <x:v>126700.05275200002</x:v>
+        <x:v>126560.434752</x:v>
       </x:c>
       <x:c r="M317" s="15" t="n">
-        <x:v>-42636.434010000004</x:v>
+        <x:v>-42776.05201000001</x:v>
       </x:c>
       <x:c r="N317" s="15" t="n">
         <x:v>1.0832932113625404</x:v>
@@ -27433,16 +27473,16 @@
         <x:v>303883.012504</x:v>
       </x:c>
       <x:c r="J345" s="15" t="n">
-        <x:v>31154.475574</x:v>
+        <x:v>31154.375574</x:v>
       </x:c>
       <x:c r="K345" s="15" t="n">
         <x:v>16648.843806</x:v>
       </x:c>
       <x:c r="L345" s="15" t="n">
-        <x:v>47803.31938</x:v>
+        <x:v>47803.21938</x:v>
       </x:c>
       <x:c r="M345" s="15" t="n">
-        <x:v>14505.631768</x:v>
+        <x:v>14505.531768</x:v>
       </x:c>
       <x:c r="N345" s="15" t="n">
         <x:v>1.390243902439034</x:v>
@@ -27758,16 +27798,16 @@
         <x:v>333999.879691</x:v>
       </x:c>
       <x:c r="J350" s="15" t="n">
-        <x:v>14072.542047</x:v>
+        <x:v>14065.246047</x:v>
       </x:c>
       <x:c r="K350" s="15" t="n">
         <x:v>20590.508965999998</x:v>
       </x:c>
       <x:c r="L350" s="15" t="n">
-        <x:v>34663.051013</x:v>
+        <x:v>34655.755013</x:v>
       </x:c>
       <x:c r="M350" s="15" t="n">
-        <x:v>-6517.966918999997</x:v>
+        <x:v>-6525.262918999997</x:v>
       </x:c>
       <x:c r="N350" s="15" t="n">
         <x:v>1.7253774263120074</x:v>
@@ -29643,16 +29683,16 @@
         <x:v>247474.979815</x:v>
       </x:c>
       <x:c r="J379" s="15" t="n">
-        <x:v>24505.47791</x:v>
+        <x:v>24481.721835</x:v>
       </x:c>
       <x:c r="K379" s="15" t="n">
         <x:v>193308.729005</x:v>
       </x:c>
       <x:c r="L379" s="15" t="n">
-        <x:v>217814.206915</x:v>
+        <x:v>217790.45084</x:v>
       </x:c>
       <x:c r="M379" s="15" t="n">
-        <x:v>-168803.251095</x:v>
+        <x:v>-168827.00717</x:v>
       </x:c>
       <x:c r="N379" s="15" t="n">
         <x:v>1.8119490695396634</x:v>
@@ -30886,7 +30926,7 @@
         <x:v>235</x:v>
       </x:c>
       <x:c r="K13" s="38" t="n">
-        <x:v>0.36086956521739133</x:v>
+        <x:v>0.41739130434782606</x:v>
       </x:c>
       <x:c r="L13" s="17" t="n">
         <x:v>229</x:v>
@@ -30962,7 +31002,7 @@
         <x:v>8916</x:v>
       </x:c>
       <x:c r="K15" s="38" t="n">
-        <x:v>0.0619876024795041</x:v>
+        <x:v>0.060187962407518496</x:v>
       </x:c>
       <x:c r="L15" s="17" t="n">
         <x:v>5000</x:v>
@@ -31000,7 +31040,7 @@
         <x:v>8916</x:v>
       </x:c>
       <x:c r="K16" s="38" t="n">
-        <x:v>0.0001999600079984003</x:v>
+        <x:v>0.0003999200159968006</x:v>
       </x:c>
       <x:c r="L16" s="17" t="n">
         <x:v>5000</x:v>
@@ -31038,7 +31078,7 @@
         <x:v>8923</x:v>
       </x:c>
       <x:c r="K17" s="38" t="n">
-        <x:v>0.1855628874225155</x:v>
+        <x:v>0.1859628074385123</x:v>
       </x:c>
       <x:c r="L17" s="17" t="n">
         <x:v>5000</x:v>
@@ -31076,7 +31116,7 @@
         <x:v>8916</x:v>
       </x:c>
       <x:c r="K18" s="38" t="n">
-        <x:v>0.2975404919016197</x:v>
+        <x:v>0.2969406118776245</x:v>
       </x:c>
       <x:c r="L18" s="17" t="n">
         <x:v>5000</x:v>
@@ -31114,7 +31154,7 @@
         <x:v>8923</x:v>
       </x:c>
       <x:c r="K19" s="38" t="n">
-        <x:v>0.42071585682863427</x:v>
+        <x:v>0.41991601679664065</x:v>
       </x:c>
       <x:c r="L19" s="17" t="n">
         <x:v>5000</x:v>
@@ -31143,16 +31183,16 @@
         <x:v>-60</x:v>
       </x:c>
       <x:c r="H20" s="42" t="n">
-        <x:v>0.041533349160342924</x:v>
+        <x:v>0.041517873773728314</x:v>
       </x:c>
       <x:c r="I20" s="42" t="n">
-        <x:v>0.02688467407060888</x:v>
+        <x:v>0.026874662141383676</x:v>
       </x:c>
       <x:c r="J20" s="17" t="n">
         <x:v>8916</x:v>
       </x:c>
       <x:c r="K20" s="38" t="n">
-        <x:v>0.0033993201359728054</x:v>
+        <x:v>0.004799040191961607</x:v>
       </x:c>
       <x:c r="L20" s="17" t="n">
         <x:v>5000</x:v>
@@ -31190,7 +31230,7 @@
         <x:v>8924</x:v>
       </x:c>
       <x:c r="K21" s="38" t="n">
-        <x:v>0.014197160567886422</x:v>
+        <x:v>0.014597080583883223</x:v>
       </x:c>
       <x:c r="L21" s="17" t="n">
         <x:v>5000</x:v>
@@ -31219,16 +31259,16 @@
         <x:v>-5</x:v>
       </x:c>
       <x:c r="H22" s="42" t="n">
-        <x:v>0.06597456875951058</x:v>
+        <x:v>0.06597707279210453</x:v>
       </x:c>
       <x:c r="I22" s="42" t="n">
-        <x:v>0.06337255176349203</x:v>
+        <x:v>0.06337007891103763</x:v>
       </x:c>
       <x:c r="J22" s="17" t="n">
         <x:v>8927</x:v>
       </x:c>
       <x:c r="K22" s="38" t="n">
-        <x:v>0.002999400119976005</x:v>
+        <x:v>0.0027994401119776045</x:v>
       </x:c>
       <x:c r="L22" s="17" t="n">
         <x:v>5000</x:v>
@@ -31266,7 +31306,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="K23" s="38" t="n">
-        <x:v>0.041666666666666664</x:v>
+        <x:v>0.20833333333333334</x:v>
       </x:c>
       <x:c r="L23" s="17" t="n">
         <x:v>23</x:v>
@@ -31304,7 +31344,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="K24" s="38" t="n">
-        <x:v>0.041666666666666664</x:v>
+        <x:v>0.7916666666666666</x:v>
       </x:c>
       <x:c r="L24" s="17" t="n">
         <x:v>23</x:v>
@@ -31342,7 +31382,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="K25" s="38" t="n">
-        <x:v>0.041666666666666664</x:v>
+        <x:v>0.7083333333333334</x:v>
       </x:c>
       <x:c r="L25" s="17" t="n">
         <x:v>23</x:v>
@@ -31380,7 +31420,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="K26" s="38" t="n">
-        <x:v>0.041666666666666664</x:v>
+        <x:v>0.7083333333333334</x:v>
       </x:c>
       <x:c r="L26" s="17" t="n">
         <x:v>23</x:v>
@@ -31418,7 +31458,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="K27" s="38" t="n">
-        <x:v>0.041666666666666664</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="L27" s="17" t="n">
         <x:v>23</x:v>
@@ -31456,7 +31496,7 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="K28" s="38" t="n">
-        <x:v>0.625</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="L28" s="17" t="n">
         <x:v>23</x:v>
@@ -31494,7 +31534,7 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="K29" s="38" t="n">
-        <x:v>0.875</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L29" s="17" t="n">
         <x:v>23</x:v>
@@ -31532,7 +31572,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="K30" s="38" t="n">
-        <x:v>0.041666666666666664</x:v>
+        <x:v>0.4166666666666667</x:v>
       </x:c>
       <x:c r="L30" s="17" t="n">
         <x:v>23</x:v>
@@ -32110,12 +32150,12 @@
     <x:mergeCell ref="A1:L2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="K5:K30">
-    <x:cfRule type="cellIs" dxfId="12" priority="1" operator="lessThanOrEqual">
+    <x:cfRule type="cellIs" dxfId="16" priority="1" operator="lessThanOrEqual">
       <x:formula>0.05</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e351ed757c34669"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc231d98453614134"/>
 </x:worksheet>
 </file>
 
@@ -39001,7 +39041,7 @@
         <x:v>-60</x:v>
       </x:c>
       <x:c r="H237" s="42" t="n">
-        <x:v>0.041533349160342924</x:v>
+        <x:v>0.041517873773728314</x:v>
       </x:c>
       <x:c r="I237" s="17" t="n">
         <x:v>8916</x:v>
@@ -39030,7 +39070,7 @@
         <x:v>-55</x:v>
       </x:c>
       <x:c r="H238" s="42" t="n">
-        <x:v>0.035931752549917394</x:v>
+        <x:v>0.035917168678208655</x:v>
       </x:c>
       <x:c r="I238" s="17" t="n">
         <x:v>8917</x:v>
@@ -39059,7 +39099,7 @@
         <x:v>-50</x:v>
       </x:c>
       <x:c r="H239" s="42" t="n">
-        <x:v>0.03436198633550965</x:v>
+        <x:v>0.03434836530694082</x:v>
       </x:c>
       <x:c r="I239" s="17" t="n">
         <x:v>8918</x:v>
@@ -39088,7 +39128,7 @@
         <x:v>-45</x:v>
       </x:c>
       <x:c r="H240" s="42" t="n">
-        <x:v>0.033352411599782604</x:v>
+        <x:v>0.033340542078802646</x:v>
       </x:c>
       <x:c r="I240" s="17" t="n">
         <x:v>8919</x:v>
@@ -39117,7 +39157,7 @@
         <x:v>-40</x:v>
       </x:c>
       <x:c r="H241" s="42" t="n">
-        <x:v>0.033298003000505366</x:v>
+        <x:v>0.03328520182040426</x:v>
       </x:c>
       <x:c r="I241" s="17" t="n">
         <x:v>8920</x:v>
@@ -39146,7 +39186,7 @@
         <x:v>-35</x:v>
       </x:c>
       <x:c r="H242" s="42" t="n">
-        <x:v>0.03182686474485637</x:v>
+        <x:v>0.031816098879456675</x:v>
       </x:c>
       <x:c r="I242" s="17" t="n">
         <x:v>8921</x:v>
@@ -39175,7 +39215,7 @@
         <x:v>-30</x:v>
       </x:c>
       <x:c r="H243" s="42" t="n">
-        <x:v>0.028071059513083356</x:v>
+        <x:v>0.02806253461309265</x:v>
       </x:c>
       <x:c r="I243" s="17" t="n">
         <x:v>8922</x:v>
@@ -39204,7 +39244,7 @@
         <x:v>-25</x:v>
       </x:c>
       <x:c r="H244" s="42" t="n">
-        <x:v>0.025962879064674753</x:v>
+        <x:v>0.02595585463826537</x:v>
       </x:c>
       <x:c r="I244" s="17" t="n">
         <x:v>8923</x:v>
@@ -39233,7 +39273,7 @@
         <x:v>-20</x:v>
       </x:c>
       <x:c r="H245" s="42" t="n">
-        <x:v>0.030025545111259957</x:v>
+        <x:v>0.030014386162482327</x:v>
       </x:c>
       <x:c r="I245" s="17" t="n">
         <x:v>8924</x:v>
@@ -39262,7 +39302,7 @@
         <x:v>-15</x:v>
       </x:c>
       <x:c r="H246" s="42" t="n">
-        <x:v>0.023993195574344362</x:v>
+        <x:v>0.02398603186386174</x:v>
       </x:c>
       <x:c r="I246" s="17" t="n">
         <x:v>8925</x:v>
@@ -39291,7 +39331,7 @@
         <x:v>-10</x:v>
       </x:c>
       <x:c r="H247" s="42" t="n">
-        <x:v>0.026194092573562082</x:v>
+        <x:v>0.026186101926444383</x:v>
       </x:c>
       <x:c r="I247" s="17" t="n">
         <x:v>8926</x:v>
@@ -39320,7 +39360,7 @@
         <x:v>-5</x:v>
       </x:c>
       <x:c r="H248" s="42" t="n">
-        <x:v>0.02749791661912031</x:v>
+        <x:v>0.02748794789598953</x:v>
       </x:c>
       <x:c r="I248" s="17" t="n">
         <x:v>8927</x:v>
@@ -39349,7 +39389,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H249" s="42" t="n">
-        <x:v>0.02688467407060888</x:v>
+        <x:v>0.026874662141383676</x:v>
       </x:c>
       <x:c r="I249" s="17" t="n">
         <x:v>8928</x:v>
@@ -39378,7 +39418,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="H250" s="42" t="n">
-        <x:v>0.025060566205264406</x:v>
+        <x:v>0.025051530317967644</x:v>
       </x:c>
       <x:c r="I250" s="17" t="n">
         <x:v>8927</x:v>
@@ -39407,7 +39447,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="H251" s="42" t="n">
-        <x:v>0.01342761998289591</x:v>
+        <x:v>0.013423552061369286</x:v>
       </x:c>
       <x:c r="I251" s="17" t="n">
         <x:v>8926</x:v>
@@ -39436,7 +39476,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="H252" s="42" t="n">
-        <x:v>0.023246198993918464</x:v>
+        <x:v>0.023239028945802872</x:v>
       </x:c>
       <x:c r="I252" s="17" t="n">
         <x:v>8925</x:v>
@@ -39465,7 +39505,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="H253" s="42" t="n">
-        <x:v>0.014526974045632824</x:v>
+        <x:v>0.014522057277257564</x:v>
       </x:c>
       <x:c r="I253" s="17" t="n">
         <x:v>8924</x:v>
@@ -39494,7 +39534,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H254" s="42" t="n">
-        <x:v>0.018406892744842814</x:v>
+        <x:v>0.018400272090308704</x:v>
       </x:c>
       <x:c r="I254" s="17" t="n">
         <x:v>8923</x:v>
@@ -39523,7 +39563,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="H255" s="42" t="n">
-        <x:v>0.013424306926772083</x:v>
+        <x:v>0.013418920238411139</x:v>
       </x:c>
       <x:c r="I255" s="17" t="n">
         <x:v>8922</x:v>
@@ -39552,7 +39592,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="H256" s="42" t="n">
-        <x:v>0.002312620491178425</x:v>
+        <x:v>0.002313021619838311</x:v>
       </x:c>
       <x:c r="I256" s="17" t="n">
         <x:v>8921</x:v>
@@ -39581,7 +39621,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="H257" s="42" t="n">
-        <x:v>0.0039200228498966405</x:v>
+        <x:v>0.00391879225850067</x:v>
       </x:c>
       <x:c r="I257" s="17" t="n">
         <x:v>8920</x:v>
@@ -39610,7 +39650,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="H258" s="42" t="n">
-        <x:v>0.011238176693130174</x:v>
+        <x:v>0.011233968294169356</x:v>
       </x:c>
       <x:c r="I258" s="17" t="n">
         <x:v>8919</x:v>
@@ -39639,7 +39679,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="H259" s="42" t="n">
-        <x:v>0.005780083296703848</x:v>
+        <x:v>0.005775660850573467</x:v>
       </x:c>
       <x:c r="I259" s="17" t="n">
         <x:v>8918</x:v>
@@ -39668,7 +39708,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="H260" s="42" t="n">
-        <x:v>0.014488139738446358</x:v>
+        <x:v>0.014482559509022167</x:v>
       </x:c>
       <x:c r="I260" s="17" t="n">
         <x:v>8917</x:v>
@@ -39697,7 +39737,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="H261" s="42" t="n">
-        <x:v>0.01602451622996063</x:v>
+        <x:v>0.016017859904978057</x:v>
       </x:c>
       <x:c r="I261" s="17" t="n">
         <x:v>8916</x:v>
@@ -40451,7 +40491,7 @@
         <x:v>-60</x:v>
       </x:c>
       <x:c r="H287" s="42" t="n">
-        <x:v>0.006649240573070573</x:v>
+        <x:v>0.006648060698092237</x:v>
       </x:c>
       <x:c r="I287" s="17" t="n">
         <x:v>8916</x:v>
@@ -40480,7 +40520,7 @@
         <x:v>-55</x:v>
       </x:c>
       <x:c r="H288" s="42" t="n">
-        <x:v>-0.00003063098834970336</x:v>
+        <x:v>-0.000030178637497983386</x:v>
       </x:c>
       <x:c r="I288" s="17" t="n">
         <x:v>8917</x:v>
@@ -40509,7 +40549,7 @@
         <x:v>-50</x:v>
       </x:c>
       <x:c r="H289" s="42" t="n">
-        <x:v>-0.018572444029987947</x:v>
+        <x:v>-0.018574028665753684</x:v>
       </x:c>
       <x:c r="I289" s="17" t="n">
         <x:v>8918</x:v>
@@ -40538,7 +40578,7 @@
         <x:v>-45</x:v>
       </x:c>
       <x:c r="H290" s="42" t="n">
-        <x:v>-0.019192947000759093</x:v>
+        <x:v>-0.01919593584949094</x:v>
       </x:c>
       <x:c r="I290" s="17" t="n">
         <x:v>8919</x:v>
@@ -40567,7 +40607,7 @@
         <x:v>-40</x:v>
       </x:c>
       <x:c r="H291" s="42" t="n">
-        <x:v>-0.006172464097191199</x:v>
+        <x:v>-0.006173514066376794</x:v>
       </x:c>
       <x:c r="I291" s="17" t="n">
         <x:v>8920</x:v>
@@ -40596,7 +40636,7 @@
         <x:v>-35</x:v>
       </x:c>
       <x:c r="H292" s="42" t="n">
-        <x:v>0.03185154047250603</x:v>
+        <x:v>0.03185227710945302</x:v>
       </x:c>
       <x:c r="I292" s="17" t="n">
         <x:v>8921</x:v>
@@ -40625,7 +40665,7 @@
         <x:v>-30</x:v>
       </x:c>
       <x:c r="H293" s="42" t="n">
-        <x:v>0.05129215728510926</x:v>
+        <x:v>0.05129603263225805</x:v>
       </x:c>
       <x:c r="I293" s="17" t="n">
         <x:v>8922</x:v>
@@ -40654,7 +40694,7 @@
         <x:v>-25</x:v>
       </x:c>
       <x:c r="H294" s="42" t="n">
-        <x:v>0.04443362067580584</x:v>
+        <x:v>0.04443185977922847</x:v>
       </x:c>
       <x:c r="I294" s="17" t="n">
         <x:v>8923</x:v>
@@ -40683,7 +40723,7 @@
         <x:v>-20</x:v>
       </x:c>
       <x:c r="H295" s="42" t="n">
-        <x:v>0.014540501373799477</x:v>
+        <x:v>0.014540059812545227</x:v>
       </x:c>
       <x:c r="I295" s="17" t="n">
         <x:v>8924</x:v>
@@ -40712,7 +40752,7 @@
         <x:v>-15</x:v>
       </x:c>
       <x:c r="H296" s="42" t="n">
-        <x:v>0.024535799846630797</x:v>
+        <x:v>0.024536335863415328</x:v>
       </x:c>
       <x:c r="I296" s="17" t="n">
         <x:v>8925</x:v>
@@ -40741,7 +40781,7 @@
         <x:v>-10</x:v>
       </x:c>
       <x:c r="H297" s="42" t="n">
-        <x:v>0.009205806016637303</x:v>
+        <x:v>0.009206816417435431</x:v>
       </x:c>
       <x:c r="I297" s="17" t="n">
         <x:v>8926</x:v>
@@ -40770,7 +40810,7 @@
         <x:v>-5</x:v>
       </x:c>
       <x:c r="H298" s="42" t="n">
-        <x:v>0.06597456875951058</x:v>
+        <x:v>0.06597707279210453</x:v>
       </x:c>
       <x:c r="I298" s="17" t="n">
         <x:v>8927</x:v>
@@ -40799,7 +40839,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H299" s="42" t="n">
-        <x:v>0.06337255176349203</x:v>
+        <x:v>0.06337007891103763</x:v>
       </x:c>
       <x:c r="I299" s="17" t="n">
         <x:v>8928</x:v>
@@ -40828,7 +40868,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="H300" s="42" t="n">
-        <x:v>0.005408245365073495</x:v>
+        <x:v>0.005405280057566731</x:v>
       </x:c>
       <x:c r="I300" s="17" t="n">
         <x:v>8927</x:v>
@@ -40857,7 +40897,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="H301" s="42" t="n">
-        <x:v>-0.005548282335628666</x:v>
+        <x:v>-0.00555485236589929</x:v>
       </x:c>
       <x:c r="I301" s="17" t="n">
         <x:v>8926</x:v>
@@ -40886,7 +40926,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="H302" s="42" t="n">
-        <x:v>0.01831308519906875</x:v>
+        <x:v>0.018312016818147203</x:v>
       </x:c>
       <x:c r="I302" s="17" t="n">
         <x:v>8925</x:v>
@@ -40915,7 +40955,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="H303" s="42" t="n">
-        <x:v>0.017304524520449026</x:v>
+        <x:v>0.0173033986903174</x:v>
       </x:c>
       <x:c r="I303" s="17" t="n">
         <x:v>8924</x:v>
@@ -40944,7 +40984,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H304" s="42" t="n">
-        <x:v>0.01010814659206796</x:v>
+        <x:v>0.010104635116446827</x:v>
       </x:c>
       <x:c r="I304" s="17" t="n">
         <x:v>8923</x:v>
@@ -40973,7 +41013,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="H305" s="42" t="n">
-        <x:v>-0.019505101162674475</x:v>
+        <x:v>-0.019529702745998155</x:v>
       </x:c>
       <x:c r="I305" s="17" t="n">
         <x:v>8922</x:v>
@@ -41002,7 +41042,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="H306" s="42" t="n">
-        <x:v>-0.012722803187272097</x:v>
+        <x:v>-0.012722477415514188</x:v>
       </x:c>
       <x:c r="I306" s="17" t="n">
         <x:v>8921</x:v>
@@ -41031,7 +41071,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="H307" s="42" t="n">
-        <x:v>-0.00015177928203081997</x:v>
+        <x:v>-0.00014302807312932254</x:v>
       </x:c>
       <x:c r="I307" s="17" t="n">
         <x:v>8920</x:v>
@@ -41060,7 +41100,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="H308" s="42" t="n">
-        <x:v>-0.007938246068143735</x:v>
+        <x:v>-0.007941239533468909</x:v>
       </x:c>
       <x:c r="I308" s="17" t="n">
         <x:v>8919</x:v>
@@ -41089,7 +41129,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="H309" s="42" t="n">
-        <x:v>-0.021302039053803123</x:v>
+        <x:v>-0.021301823297296896</x:v>
       </x:c>
       <x:c r="I309" s="17" t="n">
         <x:v>8918</x:v>
@@ -41118,7 +41158,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="H310" s="42" t="n">
-        <x:v>-0.018981738548021244</x:v>
+        <x:v>-0.0189774389003043</x:v>
       </x:c>
       <x:c r="I310" s="17" t="n">
         <x:v>8917</x:v>
@@ -41147,7 +41187,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="H311" s="42" t="n">
-        <x:v>-0.006011497326326963</x:v>
+        <x:v>-0.006011410178642371</x:v>
       </x:c>
       <x:c r="I311" s="17" t="n">
         <x:v>8916</x:v>
@@ -47206,7 +47246,7 @@
     <x:mergeCell ref="A16:H19"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb169fc806d74bfa"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08fdd51b5980491d"/>
 </x:worksheet>
 </file>
 
@@ -48004,7 +48044,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R360502820cb8478a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R256f47f1793e4d59"/>
 </x:worksheet>
 </file>
 
@@ -49636,12 +49676,12 @@
     <x:mergeCell ref="A1:N2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A5:N34">
-    <x:cfRule type="expression" dxfId="9" priority="1">
+    <x:cfRule type="expression" dxfId="13" priority="1">
       <x:formula>$A5="event"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32fad1e41ad74f1c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6586766dcdc4c0e"/>
 </x:worksheet>
 </file>
 
@@ -49739,13 +49779,13 @@
         <x:v>-1063.734002</x:v>
       </x:c>
       <x:c r="I2" s="14" t="n">
-        <x:v>14072.542047</x:v>
+        <x:v>14065.246047</x:v>
       </x:c>
       <x:c r="J2" s="14" t="n">
         <x:v>20590.508966</x:v>
       </x:c>
       <x:c r="K2" s="14" t="n">
-        <x:v>-6517.966919</x:v>
+        <x:v>-6525.262919</x:v>
       </x:c>
       <x:c r="L2" s="21" t="n">
         <x:v>0.01725377426312006</x:v>
@@ -50397,13 +50437,13 @@
         <x:v>-13847.587468</x:v>
       </x:c>
       <x:c r="I16" s="15" t="n">
-        <x:v>192860.572805</x:v>
+        <x:v>192829.510805</x:v>
       </x:c>
       <x:c r="J16" s="15" t="n">
         <x:v>121608.992469</x:v>
       </x:c>
       <x:c r="K16" s="15" t="n">
-        <x:v>71251.580336</x:v>
+        <x:v>71220.518336</x:v>
       </x:c>
       <x:c r="L16" s="22" t="n">
         <x:v>0.04461942257217848</x:v>
@@ -50444,13 +50484,13 @@
         <x:v>-9390.347911</x:v>
       </x:c>
       <x:c r="I17" s="15" t="n">
-        <x:v>57051.872186</x:v>
+        <x:v>57010.456186</x:v>
       </x:c>
       <x:c r="J17" s="15" t="n">
         <x:v>43795.551923</x:v>
       </x:c>
       <x:c r="K17" s="15" t="n">
-        <x:v>13256.320263</x:v>
+        <x:v>13214.904263</x:v>
       </x:c>
       <x:c r="L17" s="22" t="n">
         <x:v>0.027182603133994246</x:v>
@@ -50867,13 +50907,13 @@
         <x:v>-347.03775</x:v>
       </x:c>
       <x:c r="I26" s="15" t="n">
-        <x:v>24326.322525</x:v>
+        <x:v>24320.312525</x:v>
       </x:c>
       <x:c r="J26" s="15" t="n">
         <x:v>18498.612218</x:v>
       </x:c>
       <x:c r="K26" s="15" t="n">
-        <x:v>5827.710307</x:v>
+        <x:v>5821.700307</x:v>
       </x:c>
       <x:c r="L26" s="22" t="n">
         <x:v>0.03150859325270528</x:v>
@@ -53594,10 +53634,10 @@
         <x:v>inj</x:v>
       </x:c>
       <x:c r="C9" s="17" t="n">
-        <x:v>558</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="D9" s="15" t="n">
-        <x:v>32122.483968</x:v>
+        <x:v>32050.005968</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -53930,10 +53970,10 @@
         <x:v>mantra</x:v>
       </x:c>
       <x:c r="C33" s="17" t="n">
-        <x:v>268</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="D33" s="15" t="n">
-        <x:v>6111.908133</x:v>
+        <x:v>6091.283133</x:v>
       </x:c>
     </x:row>
     <x:row r="34">

</xml_diff>